<commit_message>
modified test cases and xml files
</commit_message>
<xml_diff>
--- a/testdata/logindata.xlsx
+++ b/testdata/logindata.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E558E4F6-A409-4A04-BE91-E6B7CF7A025F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{368F5521-1813-491F-A1B3-0A66486EBE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{CAAA0672-7FC0-4B22-8C0C-AC8D1F7002E2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CAAA0672-7FC0-4B22-8C0C-AC8D1F7002E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,15 +15,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -483,7 +474,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>